<commit_message>
[Dev] ScoringInfo - Edit - 更新匯入Excel範本
</commit_message>
<xml_diff>
--- a/Platform/Platform.WebSite/ModuleResources/Other/SPA_ScoringInfo/ImportTemplates/人力盤點頁籤匯入明細匯入範本.xlsx
+++ b/Platform/Platform.WebSite/ModuleResources/Other/SPA_ScoringInfo/ImportTemplates/人力盤點頁籤匯入明細匯入範本.xlsx
@@ -1,11 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr defaultThemeVersion="202300"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{6B08E27B-C996-4BDA-872F-975794FF53FD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\212486\Desktop\供應商評鑑系統\SPA系統優化2.0\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6C429A94-3C0A-4D93-8DE3-8E4C6E54E63B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1470" yWindow="1470" windowWidth="17475" windowHeight="11070" xr2:uid="{2984F46C-2D94-4B4A-AD03-55CBAB69B2C2}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{2984F46C-2D94-4B4A-AD03-55CBAB69B2C2}"/>
   </bookViews>
   <sheets>
     <sheet name="人力盤點" sheetId="1" r:id="rId1"/>
@@ -25,56 +30,142 @@
 <file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
 <comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
   <authors>
-    <author>tc={880087B3-A246-4E59-AA08-7A1066A936DB}</author>
-    <author>tc={2C2E8A0C-9DA4-4412-868B-BF14B0FFFEB7}</author>
-    <author>tc={37F7609B-BC02-4817-900E-6CE61AB69914}</author>
-    <author>tc={2014A03D-D75A-4CF8-8C28-D9D435EBA366}</author>
-    <author>tc={04F6423E-5BB4-4118-840A-6CBBE448D9C2}</author>
-    <author>tc={5B0FE75A-E067-47B0-8423-0306E6EB7324}</author>
-    <author>tc={20E0F74E-20B1-43FA-AC29-D5EDB64E837F}</author>
+    <author>tc={B5DB02D2-C399-49E7-B7C4-E85B5E50A05C}</author>
+    <author>tc={793674A0-64AC-40EA-9927-DD0ECDEBE525}</author>
+    <author>tc={DB944ABC-CC98-46D3-B2DC-C6642CB0A580}</author>
+    <author>tc={40D6F7DD-EDB0-48D7-BF2E-2B4F2E5A46EB}</author>
+    <author>tc={214B5117-D96D-4C7E-84D7-7B97FF9A3D8D}</author>
+    <author>tc={16DAE799-E688-4F0F-82D9-98A57432CE67}</author>
+    <author>tc={CAFA3218-A3D3-4CA8-8E0A-97735DB01584}</author>
+    <author>tc={C57C80AE-5C8A-40E2-A00B-DFFF3AB8C900}</author>
+    <author>tc={C0CCE8A2-1E10-4D9C-9E52-49BF415974D6}</author>
+    <author>tc={B1F6F5FE-A9A7-4B64-AF6F-D8467FC1924F}</author>
+    <author>tc={75A4EE07-6900-4089-9C3C-6761DAF7938D}</author>
+    <author>tc={BDDF9518-41F0-4531-BEDC-CC48D51170EB}</author>
+    <author>tc={DD82A34F-CD31-426D-A870-A91B0B71DC75}</author>
+    <author>tc={7993C50A-D76E-443C-A995-01118CFF7DF4}</author>
+    <author>tc={5C857AD4-A878-4389-9E10-46E74AA3A119}</author>
+    <author>tc={56A31AC6-03A9-4330-AB4F-7271C93312BA}</author>
   </authors>
   <commentList>
-    <comment ref="F1" authorId="0" shapeId="0" xr:uid="{880087B3-A246-4E59-AA08-7A1066A936DB}">
-      <text>
-        <t>[對話串註解]
-您的 Excel 版本可讓您讀取此對話串註解; 但若以較新的 Excel 版本開啟此檔案，將會移除對它進行的所有編輯。深入了解: https://go.microsoft.com/fwlink/?linkid=870924。
-註解:
-    請輸入"前期匯入" 或 "本期新增"</t>
-      </text>
-    </comment>
-    <comment ref="G1" authorId="1" shapeId="0" xr:uid="{2C2E8A0C-9DA4-4412-868B-BF14B0FFFEB7}">
-      <text>
-        <t>[對話串註解]
-您的 Excel 版本可讓您讀取此對話串註解; 但若以較新的 Excel 版本開啟此檔案，將會移除對它進行的所有編輯。深入了解: https://go.microsoft.com/fwlink/?linkid=870924。
-註解:
-    請輸入"本社社員" 或 "協力廠商"</t>
-      </text>
-    </comment>
-    <comment ref="J1" authorId="2" shapeId="0" xr:uid="{37F7609B-BC02-4817-900E-6CE61AB69914}">
-      <text>
-        <t>[對話串註解]
-您的 Excel 版本可讓您讀取此對話串註解; 但若以較新的 Excel 版本開啟此檔案，將會移除對它進行的所有編輯。深入了解: https://go.microsoft.com/fwlink/?linkid=870924。
-註解:
-    請輸入"間接"、"FE"、"PM"、"FE+PM"、"T0"、"T1"、"T2"、"T0+T1"、"T1+T2" 或 "T0+T1+T2"</t>
-      </text>
-    </comment>
-    <comment ref="K1" authorId="3" shapeId="0" xr:uid="{2014A03D-D75A-4CF8-8C28-D9D435EBA366}">
-      <text>
-        <t>[對話串註解]
-您的 Excel 版本可讓您讀取此對話串註解; 但若以較新的 Excel 版本開啟此檔案，將會移除對它進行的所有編輯。深入了解: https://go.microsoft.com/fwlink/?linkid=870924。
-註解:
-    請輸入"O"、"X" 或 "NA"</t>
-      </text>
-    </comment>
-    <comment ref="M1" authorId="4" shapeId="0" xr:uid="{04F6423E-5BB4-4118-840A-6CBBE448D9C2}">
-      <text>
-        <t>[對話串註解]
-您的 Excel 版本可讓您讀取此對話串註解; 但若以較新的 Excel 版本開啟此檔案，將會移除對它進行的所有編輯。深入了解: https://go.microsoft.com/fwlink/?linkid=870924。
-註解:
-    請輸入"新進"、"在職"、"離職" 或"其他"</t>
-      </text>
-    </comment>
-    <comment ref="N1" authorId="5" shapeId="0" xr:uid="{5B0FE75A-E067-47B0-8423-0306E6EB7324}">
+    <comment ref="A1" authorId="0" shapeId="0" xr:uid="{B5DB02D2-C399-49E7-B7C4-E85B5E50A05C}">
+      <text>
+        <t>[對話串註解]
+您的 Excel 版本可讓您讀取此對話串註解; 但若以較新的 Excel 版本開啟此檔案，將會移除對它進行的所有編輯。深入了解: https://go.microsoft.com/fwlink/?linkid=870924。
+註解:
+    須與系統上的評鑑期間一致</t>
+      </text>
+    </comment>
+    <comment ref="B1" authorId="1" shapeId="0" xr:uid="{793674A0-64AC-40EA-9927-DD0ECDEBE525}">
+      <text>
+        <t>[對話串註解]
+您的 Excel 版本可讓您讀取此對話串註解; 但若以較新的 Excel 版本開啟此檔案，將會移除對它進行的所有編輯。深入了解: https://go.microsoft.com/fwlink/?linkid=870924。
+註解:
+    須與系統上的評鑑單位一致</t>
+      </text>
+    </comment>
+    <comment ref="C1" authorId="2" shapeId="0" xr:uid="{DB944ABC-CC98-46D3-B2DC-C6642CB0A580}">
+      <text>
+        <t>[對話串註解]
+您的 Excel 版本可讓您讀取此對話串註解; 但若以較新的 Excel 版本開啟此檔案，將會移除對它進行的所有編輯。深入了解: https://go.microsoft.com/fwlink/?linkid=870924。
+註解:
+    須與系統上的服務對象一致</t>
+      </text>
+    </comment>
+    <comment ref="D1" authorId="3" shapeId="0" xr:uid="{40D6F7DD-EDB0-48D7-BF2E-2B4F2E5A46EB}">
+      <text>
+        <t>[對話串註解]
+您的 Excel 版本可讓您讀取此對話串註解; 但若以較新的 Excel 版本開啟此檔案，將會移除對它進行的所有編輯。深入了解: https://go.microsoft.com/fwlink/?linkid=870924。
+註解:
+    須與系統上的評鑑項目一致</t>
+      </text>
+    </comment>
+    <comment ref="E1" authorId="4" shapeId="0" xr:uid="{214B5117-D96D-4C7E-84D7-7B97FF9A3D8D}">
+      <text>
+        <t>[對話串註解]
+您的 Excel 版本可讓您讀取此對話串註解; 但若以較新的 Excel 版本開啟此檔案，將會移除對它進行的所有編輯。深入了解: https://go.microsoft.com/fwlink/?linkid=870924。
+註解:
+    須與系統上的受評供應商一致</t>
+      </text>
+    </comment>
+    <comment ref="F1" authorId="5" shapeId="0" xr:uid="{16DAE799-E688-4F0F-82D9-98A57432CE67}">
+      <text>
+        <t>[對話串註解]
+您的 Excel 版本可讓您讀取此對話串註解; 但若以較新的 Excel 版本開啟此檔案，將會移除對它進行的所有編輯。深入了解: https://go.microsoft.com/fwlink/?linkid=870924。
+註解:
+    前期既有人員，填"前期匯入" 
+新增人員，填 "本期新增"</t>
+      </text>
+    </comment>
+    <comment ref="G1" authorId="6" shapeId="0" xr:uid="{CAFA3218-A3D3-4CA8-8E0A-97735DB01584}">
+      <text>
+        <t>[對話串註解]
+您的 Excel 版本可讓您讀取此對話串註解; 但若以較新的 Excel 版本開啟此檔案，將會移除對它進行的所有編輯。深入了解: https://go.microsoft.com/fwlink/?linkid=870924。
+註解:
+    員工隸屬之供應商(本社)，或供應商之協力廠商
+請填 "本社社員" 或 "協力廠商"</t>
+      </text>
+    </comment>
+    <comment ref="H1" authorId="7" shapeId="0" xr:uid="{C57C80AE-5C8A-40E2-A00B-DFFF3AB8C900}">
+      <text>
+        <t>[對話串註解]
+您的 Excel 版本可讓您讀取此對話串註解; 但若以較新的 Excel 版本開啟此檔案，將會移除對它進行的所有編輯。深入了解: https://go.microsoft.com/fwlink/?linkid=870924。
+註解:
+    員工隸屬之供應商名稱；
+若為本社社員，填寫同受評供應商；
+若社員為供應商之協力廠商，填協力廠商名稱</t>
+      </text>
+    </comment>
+    <comment ref="I1" authorId="8" shapeId="0" xr:uid="{C0CCE8A2-1E10-4D9C-9E52-49BF415974D6}">
+      <text>
+        <t>[對話串註解]
+您的 Excel 版本可讓您讀取此對話串註解; 但若以較新的 Excel 版本開啟此檔案，將會移除對它進行的所有編輯。深入了解: https://go.microsoft.com/fwlink/?linkid=870924。
+註解:
+    供應商之協力廠商之員工姓名</t>
+      </text>
+    </comment>
+    <comment ref="J1" authorId="9" shapeId="0" xr:uid="{B1F6F5FE-A9A7-4B64-AF6F-D8467FC1924F}">
+      <text>
+        <t>[對話串註解]
+您的 Excel 版本可讓您讀取此對話串註解; 但若以較新的 Excel 版本開啟此檔案，將會移除對它進行的所有編輯。深入了解: https://go.microsoft.com/fwlink/?linkid=870924。
+註解:
+    評鑑期間主要負責作業
+評鑑項目=safety不用填寫
+請輸入"間接"、"FE"、"PM"、"FE+PM"、"T0"、"T1"、"T2"、"T0+T1"、"T1+T2" 或 "T0+T1+T2"</t>
+      </text>
+    </comment>
+    <comment ref="K1" authorId="10" shapeId="0" xr:uid="{75A4EE07-6900-4089-9C3C-6761DAF7938D}">
+      <text>
+        <t xml:space="preserve">[對話串註解]
+您的 Excel 版本可讓您讀取此對話串註解; 但若以較新的 Excel 版本開啟此檔案，將會移除對它進行的所有編輯。深入了解: https://go.microsoft.com/fwlink/?linkid=870924。
+註解:
+    評鑑項目=safety不用填寫
+能獨立作業，填"O"；
+不能獨立作業，填"X" ；
+間接作業，填 "NA"
+（大小寫必須完全一致) </t>
+      </text>
+    </comment>
+    <comment ref="L1" authorId="11" shapeId="0" xr:uid="{BDDF9518-41F0-4531-BEDC-CC48D51170EB}">
+      <text>
+        <t>[對話串註解]
+您的 Excel 版本可讓您讀取此對話串註解; 但若以較新的 Excel 版本開啟此檔案，將會移除對它進行的所有編輯。深入了解: https://go.microsoft.com/fwlink/?linkid=870924。
+註解:
+    由管理者對人員的[主要負責作業]熟練度來判定等級
+評鑑項目=Safety不用填寫</t>
+      </text>
+    </comment>
+    <comment ref="M1" authorId="12" shapeId="0" xr:uid="{DD82A34F-CD31-426D-A870-A91B0B71DC75}">
+      <text>
+        <t>[對話串註解]
+您的 Excel 版本可讓您讀取此對話串註解; 但若以較新的 Excel 版本開啟此檔案，將會移除對它進行的所有編輯。深入了解: https://go.microsoft.com/fwlink/?linkid=870924。
+註解:
+    請輸入"新進"、"在職"、"離職" 或"其他"
+1. 資料來源是本期新增，只能填"新進" 或"其他"
+2. 資料來源是前期匯入，"在職"、"離職" 或"其他"</t>
+      </text>
+    </comment>
+    <comment ref="N1" authorId="13" shapeId="0" xr:uid="{7993C50A-D76E-443C-A995-01118CFF7DF4}">
       <text>
         <t>[對話串註解]
 您的 Excel 版本可讓您讀取此對話串註解; 但若以較新的 Excel 版本開啟此檔案，將會移除對它進行的所有編輯。深入了解: https://go.microsoft.com/fwlink/?linkid=870924。
@@ -82,12 +173,20 @@
     請輸入數字</t>
       </text>
     </comment>
-    <comment ref="O1" authorId="6" shapeId="0" xr:uid="{20E0F74E-20B1-43FA-AC29-D5EDB64E837F}">
+    <comment ref="O1" authorId="14" shapeId="0" xr:uid="{5C857AD4-A878-4389-9E10-46E74AA3A119}">
       <text>
         <t>[對話串註解]
 您的 Excel 版本可讓您讀取此對話串註解; 但若以較新的 Excel 版本開啟此檔案，將會移除對它進行的所有編輯。深入了解: https://go.microsoft.com/fwlink/?linkid=870924。
 註解:
     請輸入0~11數字</t>
+      </text>
+    </comment>
+    <comment ref="P1" authorId="15" shapeId="0" xr:uid="{56A31AC6-03A9-4330-AB4F-7271C93312BA}">
+      <text>
+        <t>[對話串註解]
+您的 Excel 版本可讓您讀取此對話串註解; 但若以較新的 Excel 版本開啟此檔案，將會移除對它進行的所有編輯。深入了解: https://go.microsoft.com/fwlink/?linkid=870924。
+註解:
+    員工狀態"其他"，請在備註說明</t>
       </text>
     </comment>
   </commentList>
@@ -165,7 +264,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3">
+  <fonts count="4">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -188,6 +287,12 @@
       <family val="2"/>
       <charset val="136"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color indexed="81"/>
+      <name val="Tahoma"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="3">
@@ -271,7 +376,7 @@
 
 <file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
 <personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <person displayName="a92573" id="{C1111D30-88A5-4DC6-9F1D-2BD2B0298372}" userId="S::a92573@e365.shop::a5c1d779-7da7-4f72-9b02-b37c31ccf028" providerId="AD"/>
+  <person displayName="TET SCM Chen, Grace" id="{8D9489BD-DFBC-42AD-AEE1-A37CD6E87A3E}" userId="S::grace2.chen@tel.com::6dbe00fd-a5fc-44db-ab99-cd07605e303e" providerId="AD"/>
 </personList>
 </file>
 
@@ -592,26 +697,66 @@
 
 <file path=xl/threadedComments/threadedComment1.xml><?xml version="1.0" encoding="utf-8"?>
 <ThreadedComments xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <threadedComment ref="F1" dT="2026-07-17T23:14:28.15" personId="{C1111D30-88A5-4DC6-9F1D-2BD2B0298372}" id="{880087B3-A246-4E59-AA08-7A1066A936DB}">
-    <text>請輸入"前期匯入" 或 "本期新增"</text>
-  </threadedComment>
-  <threadedComment ref="G1" dT="2026-07-17T23:15:12.90" personId="{C1111D30-88A5-4DC6-9F1D-2BD2B0298372}" id="{2C2E8A0C-9DA4-4412-868B-BF14B0FFFEB7}">
-    <text>請輸入"本社社員" 或 "協力廠商"</text>
-  </threadedComment>
-  <threadedComment ref="J1" dT="2026-07-17T23:41:12.40" personId="{C1111D30-88A5-4DC6-9F1D-2BD2B0298372}" id="{37F7609B-BC02-4817-900E-6CE61AB69914}">
-    <text>請輸入"間接"、"FE"、"PM"、"FE+PM"、"T0"、"T1"、"T2"、"T0+T1"、"T1+T2" 或 "T0+T1+T2"</text>
-  </threadedComment>
-  <threadedComment ref="K1" dT="2026-07-17T23:36:44.75" personId="{C1111D30-88A5-4DC6-9F1D-2BD2B0298372}" id="{2014A03D-D75A-4CF8-8C28-D9D435EBA366}">
-    <text>請輸入"O"、"X" 或 "NA"</text>
-  </threadedComment>
-  <threadedComment ref="M1" dT="2026-07-17T23:37:43.64" personId="{C1111D30-88A5-4DC6-9F1D-2BD2B0298372}" id="{04F6423E-5BB4-4118-840A-6CBBE448D9C2}">
-    <text>請輸入"新進"、"在職"、"離職" 或"其他"</text>
-  </threadedComment>
-  <threadedComment ref="N1" dT="2026-07-17T23:38:25.09" personId="{C1111D30-88A5-4DC6-9F1D-2BD2B0298372}" id="{5B0FE75A-E067-47B0-8423-0306E6EB7324}">
+  <threadedComment ref="A1" dT="2026-09-17T02:57:37.00" personId="{8D9489BD-DFBC-42AD-AEE1-A37CD6E87A3E}" id="{B5DB02D2-C399-49E7-B7C4-E85B5E50A05C}">
+    <text>須與系統上的評鑑期間一致</text>
+  </threadedComment>
+  <threadedComment ref="B1" dT="2026-09-17T02:57:51.28" personId="{8D9489BD-DFBC-42AD-AEE1-A37CD6E87A3E}" id="{793674A0-64AC-40EA-9927-DD0ECDEBE525}">
+    <text>須與系統上的評鑑單位一致</text>
+  </threadedComment>
+  <threadedComment ref="C1" dT="2026-09-17T02:58:14.38" personId="{8D9489BD-DFBC-42AD-AEE1-A37CD6E87A3E}" id="{DB944ABC-CC98-46D3-B2DC-C6642CB0A580}">
+    <text>須與系統上的服務對象一致</text>
+  </threadedComment>
+  <threadedComment ref="D1" dT="2026-09-17T02:58:34.54" personId="{8D9489BD-DFBC-42AD-AEE1-A37CD6E87A3E}" id="{40D6F7DD-EDB0-48D7-BF2E-2B4F2E5A46EB}">
+    <text>須與系統上的評鑑項目一致</text>
+  </threadedComment>
+  <threadedComment ref="E1" dT="2026-09-17T02:58:57.50" personId="{8D9489BD-DFBC-42AD-AEE1-A37CD6E87A3E}" id="{214B5117-D96D-4C7E-84D7-7B97FF9A3D8D}">
+    <text>須與系統上的受評供應商一致</text>
+  </threadedComment>
+  <threadedComment ref="F1" dT="2026-09-22T08:05:53.04" personId="{8D9489BD-DFBC-42AD-AEE1-A37CD6E87A3E}" id="{16DAE799-E688-4F0F-82D9-98A57432CE67}">
+    <text>前期既有人員，填"前期匯入" 
+新增人員，填 "本期新增"</text>
+  </threadedComment>
+  <threadedComment ref="G1" dT="2026-09-22T07:56:15.70" personId="{8D9489BD-DFBC-42AD-AEE1-A37CD6E87A3E}" id="{CAFA3218-A3D3-4CA8-8E0A-97735DB01584}">
+    <text>員工隸屬之供應商(本社)，或供應商之協力廠商
+請填 "本社社員" 或 "協力廠商"</text>
+  </threadedComment>
+  <threadedComment ref="H1" dT="2026-09-22T07:58:55.59" personId="{8D9489BD-DFBC-42AD-AEE1-A37CD6E87A3E}" id="{C57C80AE-5C8A-40E2-A00B-DFFF3AB8C900}">
+    <text>員工隸屬之供應商名稱；
+若為本社社員，填寫同受評供應商；
+若社員為供應商之協力廠商，填協力廠商名稱</text>
+  </threadedComment>
+  <threadedComment ref="I1" dT="2026-09-22T08:16:09.52" personId="{8D9489BD-DFBC-42AD-AEE1-A37CD6E87A3E}" id="{C0CCE8A2-1E10-4D9C-9E52-49BF415974D6}">
+    <text>供應商之協力廠商之員工姓名</text>
+  </threadedComment>
+  <threadedComment ref="J1" dT="2026-09-22T08:01:36.57" personId="{8D9489BD-DFBC-42AD-AEE1-A37CD6E87A3E}" id="{B1F6F5FE-A9A7-4B64-AF6F-D8467FC1924F}">
+    <text>評鑑期間主要負責作業
+評鑑項目=safety不用填寫
+請輸入"間接"、"FE"、"PM"、"FE+PM"、"T0"、"T1"、"T2"、"T0+T1"、"T1+T2" 或 "T0+T1+T2"</text>
+  </threadedComment>
+  <threadedComment ref="K1" dT="2026-09-22T08:03:01.46" personId="{8D9489BD-DFBC-42AD-AEE1-A37CD6E87A3E}" id="{75A4EE07-6900-4089-9C3C-6761DAF7938D}">
+    <text xml:space="preserve">評鑑項目=safety不用填寫
+能獨立作業，填"O"；
+不能獨立作業，填"X" ；
+間接作業，填 "NA"
+（大小寫必須完全一致) </text>
+  </threadedComment>
+  <threadedComment ref="L1" dT="2026-09-22T08:24:02.19" personId="{8D9489BD-DFBC-42AD-AEE1-A37CD6E87A3E}" id="{BDDF9518-41F0-4531-BEDC-CC48D51170EB}">
+    <text>由管理者對人員的[主要負責作業]熟練度來判定等級
+評鑑項目=Safety不用填寫</text>
+  </threadedComment>
+  <threadedComment ref="M1" dT="2026-09-22T08:27:58.24" personId="{8D9489BD-DFBC-42AD-AEE1-A37CD6E87A3E}" id="{DD82A34F-CD31-426D-A870-A91B0B71DC75}">
+    <text>請輸入"新進"、"在職"、"離職" 或"其他"
+1. 資料來源是本期新增，只能填"新進" 或"其他"
+2. 資料來源是前期匯入，"在職"、"離職" 或"其他"</text>
+  </threadedComment>
+  <threadedComment ref="N1" dT="2026-09-22T08:29:46.52" personId="{8D9489BD-DFBC-42AD-AEE1-A37CD6E87A3E}" id="{7993C50A-D76E-443C-A995-01118CFF7DF4}">
     <text>請輸入數字</text>
   </threadedComment>
-  <threadedComment ref="O1" dT="2026-07-17T23:38:13.68" personId="{C1111D30-88A5-4DC6-9F1D-2BD2B0298372}" id="{20E0F74E-20B1-43FA-AC29-D5EDB64E837F}">
+  <threadedComment ref="O1" dT="2026-09-22T08:30:14.81" personId="{8D9489BD-DFBC-42AD-AEE1-A37CD6E87A3E}" id="{5C857AD4-A878-4389-9E10-46E74AA3A119}">
     <text>請輸入0~11數字</text>
+  </threadedComment>
+  <threadedComment ref="P1" dT="2026-09-23T06:38:31.39" personId="{8D9489BD-DFBC-42AD-AEE1-A37CD6E87A3E}" id="{56A31AC6-03A9-4330-AB4F-7271C93312BA}">
+    <text>員工狀態"其他"，請在備註說明</text>
   </threadedComment>
 </ThreadedComments>
 </file>
@@ -621,11 +766,11 @@
   <dimension ref="A1:P1"/>
   <sheetFormatPr defaultRowHeight="18" customHeight="1"/>
   <cols>
-    <col min="1" max="12" width="15.796875" customWidth="1"/>
-    <col min="13" max="16" width="25.796875" customWidth="1"/>
+    <col min="1" max="12" width="15.81640625" customWidth="1"/>
+    <col min="13" max="16" width="25.81640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" ht="28.8" customHeight="1">
+    <row r="1" spans="1:16" ht="28.75" customHeight="1">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>

</xml_diff>